<commit_message>
Updated Portfolio Management Plan
</commit_message>
<xml_diff>
--- a/financial_models/Stock_Monitor.xlsx
+++ b/financial_models/Stock_Monitor.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jerry\PycharmProjects\Invest_Proc_v4\financial_models\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6416A34F-80DA-46A4-A23A-C31591A75733}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D51AEC07-4EE0-4CA7-ACAF-E84B8CAB220C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="33720" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1344,6 +1344,135 @@
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
   <si>
+    <t>Imported from Valuation models to Opportunities Sheet</t>
+    <phoneticPr fontId="17" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <i/>
+        <sz val="9"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">Process: </t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="9"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>Calculate a Risk Appetite Score (0–8 scale) using four market indicators to set cash reserves.</t>
+    </r>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Strategic reserve for strategic opportunities.</t>
+    <phoneticPr fontId="17" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <i/>
+        <sz val="9"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">Objective: </t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="9"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>Determine the optimal capital allocation at current market prices, while reserving capital for strategic deployment.</t>
+    </r>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>3. Allocation Weight:</t>
+    <phoneticPr fontId="17" type="noConversion"/>
+  </si>
+  <si>
+    <t>allocation_weight_i = provisional_weight_i * (1-Δweight_i)</t>
+    <phoneticPr fontId="17" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <t>allocated_weight = Σ</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color theme="1"/>
+        <rFont val="Microsoft YaHei UI"/>
+        <family val="2"/>
+        <charset val="134"/>
+      </rPr>
+      <t>(</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>allocation_weight_i)</t>
+    </r>
+    <phoneticPr fontId="17" type="noConversion"/>
+  </si>
+  <si>
+    <t>Return = Σ(allocation_weight_i× R_i) + (Projected Cash % × Cash Yield)</t>
+    <phoneticPr fontId="17" type="noConversion"/>
+  </si>
+  <si>
+    <t>Allocation Weight</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>4. Total Allocated Weight:</t>
+    <phoneticPr fontId="17" type="noConversion"/>
+  </si>
+  <si>
+    <t>Calculate Allocation Weight (Data Processing)</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <i/>
+        <sz val="9"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>Total investable capital Consideration:</t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="9"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> This issue will be resolved at processing the Total Allocated Weight.</t>
+    </r>
+    <phoneticPr fontId="17" type="noConversion"/>
+  </si>
+  <si>
     <r>
       <rPr>
         <b/>
@@ -1363,136 +1492,7 @@
         <rFont val="Arial"/>
         <family val="2"/>
       </rPr>
-      <t>When the Projected Portfolio Return falls below the benchmark, it is due to overly conservative cash reserve settings or a lack of eligible opportunities. Corrective action is needed to address these issues.</t>
-    </r>
-    <phoneticPr fontId="17" type="noConversion"/>
-  </si>
-  <si>
-    <t>Imported from Valuation models to Opportunities Sheet</t>
-    <phoneticPr fontId="17" type="noConversion"/>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <b/>
-        <i/>
-        <sz val="9"/>
-        <color theme="1"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">Process: </t>
-    </r>
-    <r>
-      <rPr>
-        <i/>
-        <sz val="9"/>
-        <color theme="1"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t>Calculate a Risk Appetite Score (0–8 scale) using four market indicators to set cash reserves.</t>
-    </r>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>Strategic reserve for strategic opportunities.</t>
-    <phoneticPr fontId="17" type="noConversion"/>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <b/>
-        <i/>
-        <sz val="9"/>
-        <color theme="1"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">Objective: </t>
-    </r>
-    <r>
-      <rPr>
-        <i/>
-        <sz val="9"/>
-        <color theme="1"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t>Determine the optimal capital allocation at current market prices, while reserving capital for strategic deployment.</t>
-    </r>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>3. Allocation Weight:</t>
-    <phoneticPr fontId="17" type="noConversion"/>
-  </si>
-  <si>
-    <t>allocation_weight_i = provisional_weight_i * (1-Δweight_i)</t>
-    <phoneticPr fontId="17" type="noConversion"/>
-  </si>
-  <si>
-    <r>
-      <t>allocated_weight = Σ</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="9"/>
-        <color theme="1"/>
-        <rFont val="Microsoft YaHei UI"/>
-        <family val="2"/>
-        <charset val="134"/>
-      </rPr>
-      <t>(</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="9"/>
-        <color theme="1"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t>allocation_weight_i)</t>
-    </r>
-    <phoneticPr fontId="17" type="noConversion"/>
-  </si>
-  <si>
-    <t>Return = Σ(allocation_weight_i× R_i) + (Projected Cash % × Cash Yield)</t>
-    <phoneticPr fontId="17" type="noConversion"/>
-  </si>
-  <si>
-    <t>Allocation Weight</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>4. Total Allocated Weight:</t>
-    <phoneticPr fontId="17" type="noConversion"/>
-  </si>
-  <si>
-    <t>Calculate Allocation Weight (Data Processing)</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <b/>
-        <i/>
-        <sz val="9"/>
-        <color theme="1"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t>Total investable capital Consideration:</t>
-    </r>
-    <r>
-      <rPr>
-        <i/>
-        <sz val="9"/>
-        <color theme="1"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve"> This issue will be resolved at processing the Total Allocated Weight.</t>
+      <t>When the Projected Portfolio Return falls below the benchmark, it is due to overly conservative cash reserve settings or a lack of eligible opportunities. Manual corrective action is needed to address these issues.</t>
     </r>
     <phoneticPr fontId="17" type="noConversion"/>
   </si>
@@ -1950,17 +1950,17 @@
     <xf numFmtId="179" fontId="26" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
     </xf>
     <xf numFmtId="4" fontId="6" fillId="5" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -2334,12 +2334,12 @@
       <c r="E2" s="21"/>
     </row>
     <row r="4" spans="1:5" ht="24.4" customHeight="1">
-      <c r="B4" s="64" t="s">
+      <c r="B4" s="65" t="s">
         <v>208</v>
       </c>
-      <c r="C4" s="64"/>
-      <c r="D4" s="64"/>
-      <c r="E4" s="64"/>
+      <c r="C4" s="65"/>
+      <c r="D4" s="65"/>
+      <c r="E4" s="65"/>
     </row>
     <row r="5" spans="1:5">
       <c r="B5" s="24" t="s">
@@ -2361,12 +2361,12 @@
       <c r="C8" s="62"/>
     </row>
     <row r="9" spans="1:5">
-      <c r="B9" s="64" t="s">
-        <v>221</v>
-      </c>
-      <c r="C9" s="64"/>
-      <c r="D9" s="64"/>
-      <c r="E9" s="64"/>
+      <c r="B9" s="65" t="s">
+        <v>220</v>
+      </c>
+      <c r="C9" s="65"/>
+      <c r="D9" s="65"/>
+      <c r="E9" s="65"/>
     </row>
     <row r="11" spans="1:5">
       <c r="B11" s="23" t="s">
@@ -2405,7 +2405,7 @@
         <v>216</v>
       </c>
       <c r="C16" s="4" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
     </row>
     <row r="17" spans="1:5">
@@ -2455,12 +2455,12 @@
     </row>
     <row r="26" spans="1:5">
       <c r="A26" s="18"/>
-      <c r="B26" s="64" t="s">
+      <c r="B26" s="65" t="s">
         <v>214</v>
       </c>
-      <c r="C26" s="64"/>
-      <c r="D26" s="64"/>
-      <c r="E26" s="64"/>
+      <c r="C26" s="65"/>
+      <c r="D26" s="65"/>
+      <c r="E26" s="65"/>
     </row>
     <row r="27" spans="1:5">
       <c r="A27" s="18"/>
@@ -2554,20 +2554,20 @@
       </c>
     </row>
     <row r="41" spans="1:5">
-      <c r="B41" s="64" t="s">
+      <c r="B41" s="65" t="s">
         <v>158</v>
       </c>
-      <c r="C41" s="64"/>
-      <c r="D41" s="64"/>
-      <c r="E41" s="64"/>
+      <c r="C41" s="65"/>
+      <c r="D41" s="65"/>
+      <c r="E41" s="65"/>
     </row>
     <row r="42" spans="1:5" ht="24.4" customHeight="1">
-      <c r="B42" s="64" t="s">
+      <c r="B42" s="65" t="s">
         <v>88</v>
       </c>
-      <c r="C42" s="64"/>
-      <c r="D42" s="64"/>
-      <c r="E42" s="64"/>
+      <c r="C42" s="65"/>
+      <c r="D42" s="65"/>
+      <c r="E42" s="65"/>
     </row>
     <row r="44" spans="1:5">
       <c r="A44" s="21" t="s">
@@ -2579,12 +2579,12 @@
       <c r="E44" s="21"/>
     </row>
     <row r="46" spans="1:5">
-      <c r="B46" s="64" t="s">
-        <v>219</v>
-      </c>
-      <c r="C46" s="64"/>
-      <c r="D46" s="64"/>
-      <c r="E46" s="64"/>
+      <c r="B46" s="65" t="s">
+        <v>218</v>
+      </c>
+      <c r="C46" s="65"/>
+      <c r="D46" s="65"/>
+      <c r="E46" s="65"/>
     </row>
     <row r="48" spans="1:5">
       <c r="B48" s="23" t="s">
@@ -2629,7 +2629,7 @@
         <v>0.2</v>
       </c>
       <c r="D53" s="63" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
       <c r="E53" s="56"/>
     </row>
@@ -2769,12 +2769,12 @@
       <c r="E71" s="21"/>
     </row>
     <row r="73" spans="1:5">
-      <c r="B73" s="64" t="s">
+      <c r="B73" s="65" t="s">
         <v>201</v>
       </c>
-      <c r="C73" s="64"/>
-      <c r="D73" s="64"/>
-      <c r="E73" s="64"/>
+      <c r="C73" s="65"/>
+      <c r="D73" s="65"/>
+      <c r="E73" s="65"/>
     </row>
     <row r="75" spans="1:5">
       <c r="A75" s="28" t="s">
@@ -2827,7 +2827,7 @@
         <v>148</v>
       </c>
       <c r="B85" s="20" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
     </row>
     <row r="86" spans="1:5">
@@ -2836,36 +2836,36 @@
       </c>
     </row>
     <row r="87" spans="1:5">
-      <c r="B87" s="67" t="s">
+      <c r="B87" s="66" t="s">
         <v>197</v>
       </c>
-      <c r="C87" s="67"/>
-      <c r="D87" s="67"/>
-      <c r="E87" s="67"/>
+      <c r="C87" s="66"/>
+      <c r="D87" s="66"/>
+      <c r="E87" s="66"/>
     </row>
     <row r="88" spans="1:5">
-      <c r="B88" s="66" t="s">
+      <c r="B88" s="64" t="s">
         <v>195</v>
       </c>
-      <c r="C88" s="66"/>
-      <c r="D88" s="66"/>
-      <c r="E88" s="66"/>
+      <c r="C88" s="64"/>
+      <c r="D88" s="64"/>
+      <c r="E88" s="64"/>
     </row>
     <row r="89" spans="1:5" ht="24.4" customHeight="1">
-      <c r="B89" s="64" t="s">
+      <c r="B89" s="65" t="s">
         <v>194</v>
       </c>
-      <c r="C89" s="64"/>
-      <c r="D89" s="64"/>
-      <c r="E89" s="64"/>
+      <c r="C89" s="65"/>
+      <c r="D89" s="65"/>
+      <c r="E89" s="65"/>
     </row>
     <row r="90" spans="1:5">
-      <c r="B90" s="64" t="s">
-        <v>229</v>
-      </c>
-      <c r="C90" s="64"/>
-      <c r="D90" s="64"/>
-      <c r="E90" s="64"/>
+      <c r="B90" s="65" t="s">
+        <v>228</v>
+      </c>
+      <c r="C90" s="65"/>
+      <c r="D90" s="65"/>
+      <c r="E90" s="65"/>
     </row>
     <row r="92" spans="1:5">
       <c r="B92" s="24" t="s">
@@ -2894,37 +2894,37 @@
     </row>
     <row r="98" spans="1:5">
       <c r="B98" s="24" t="s">
+        <v>221</v>
+      </c>
+    </row>
+    <row r="99" spans="1:5">
+      <c r="B99" s="67" t="s">
         <v>222</v>
       </c>
-    </row>
-    <row r="99" spans="1:5">
-      <c r="B99" s="65" t="s">
-        <v>223</v>
-      </c>
-      <c r="C99" s="65"/>
-      <c r="D99" s="65"/>
-      <c r="E99" s="65"/>
+      <c r="C99" s="67"/>
+      <c r="D99" s="67"/>
+      <c r="E99" s="67"/>
     </row>
     <row r="101" spans="1:5">
       <c r="B101" s="24" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
     </row>
     <row r="102" spans="1:5" ht="12.4">
-      <c r="B102" s="65" t="s">
-        <v>224</v>
-      </c>
-      <c r="C102" s="65"/>
-      <c r="D102" s="65"/>
-      <c r="E102" s="65"/>
+      <c r="B102" s="67" t="s">
+        <v>223</v>
+      </c>
+      <c r="C102" s="67"/>
+      <c r="D102" s="67"/>
+      <c r="E102" s="67"/>
     </row>
     <row r="103" spans="1:5" ht="24.4" customHeight="1">
-      <c r="B103" s="64" t="s">
+      <c r="B103" s="65" t="s">
         <v>215</v>
       </c>
-      <c r="C103" s="64"/>
-      <c r="D103" s="64"/>
-      <c r="E103" s="64"/>
+      <c r="C103" s="65"/>
+      <c r="D103" s="65"/>
+      <c r="E103" s="65"/>
     </row>
     <row r="105" spans="1:5">
       <c r="A105" s="28" t="s">
@@ -2951,7 +2951,7 @@
     </row>
     <row r="110" spans="1:5">
       <c r="B110" s="1" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
     </row>
     <row r="112" spans="1:5">
@@ -2972,20 +2972,20 @@
         <v>181</v>
       </c>
       <c r="C114" s="44">
-        <v>0.10199999999999999</v>
+        <v>0.13</v>
       </c>
       <c r="D114" s="62" t="str">
-        <f>IF(C114&lt;benchmark,"Warning: Return is lower than the Benchmark.")</f>
-        <v>Warning: Return is lower than the Benchmark.</v>
+        <f>IF(C114&lt;benchmark,"Warning: Return is lower than the Benchmark.","")</f>
+        <v/>
       </c>
     </row>
     <row r="116" spans="1:5" ht="24.4" customHeight="1">
-      <c r="B116" s="64" t="s">
-        <v>217</v>
-      </c>
-      <c r="C116" s="64"/>
-      <c r="D116" s="64"/>
-      <c r="E116" s="64"/>
+      <c r="B116" s="65" t="s">
+        <v>229</v>
+      </c>
+      <c r="C116" s="65"/>
+      <c r="D116" s="65"/>
+      <c r="E116" s="65"/>
     </row>
     <row r="118" spans="1:5">
       <c r="A118" s="21" t="s">
@@ -3018,6 +3018,12 @@
     </row>
   </sheetData>
   <mergeCells count="15">
+    <mergeCell ref="B116:E116"/>
+    <mergeCell ref="B99:E99"/>
+    <mergeCell ref="B102:E102"/>
+    <mergeCell ref="B103:E103"/>
+    <mergeCell ref="B89:E89"/>
+    <mergeCell ref="B90:E90"/>
     <mergeCell ref="B88:E88"/>
     <mergeCell ref="B73:E73"/>
     <mergeCell ref="B87:E87"/>
@@ -3027,12 +3033,6 @@
     <mergeCell ref="B26:E26"/>
     <mergeCell ref="B41:E41"/>
     <mergeCell ref="B42:E42"/>
-    <mergeCell ref="B116:E116"/>
-    <mergeCell ref="B99:E99"/>
-    <mergeCell ref="B102:E102"/>
-    <mergeCell ref="B103:E103"/>
-    <mergeCell ref="B89:E89"/>
-    <mergeCell ref="B90:E90"/>
   </mergeCells>
   <phoneticPr fontId="17" type="noConversion"/>
   <pageMargins left="0.25" right="0.25" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -3116,7 +3116,7 @@
         <v>62</v>
       </c>
       <c r="I2" s="7" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="J2" s="8" t="s">
         <v>8</v>
@@ -5743,15 +5743,15 @@
       <c r="B5" s="74" t="s">
         <v>108</v>
       </c>
-      <c r="C5" s="65"/>
-      <c r="D5" s="65"/>
+      <c r="C5" s="67"/>
+      <c r="D5" s="67"/>
     </row>
     <row r="6" spans="1:4">
       <c r="B6" s="74" t="s">
         <v>109</v>
       </c>
-      <c r="C6" s="65"/>
-      <c r="D6" s="65"/>
+      <c r="C6" s="67"/>
+      <c r="D6" s="67"/>
     </row>
     <row r="8" spans="1:4">
       <c r="B8" s="1" t="s">

</xml_diff>

<commit_message>
Updated models or Monitor
</commit_message>
<xml_diff>
--- a/financial_models/Stock_Monitor.xlsx
+++ b/financial_models/Stock_Monitor.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jerry\PycharmProjects\Invest_Proc_v4\financial_models\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D51AEC07-4EE0-4CA7-ACAF-E84B8CAB220C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E3BC3333-5B2A-4F36-BB10-7F3AAAFEF0DE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="33720" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="17115" windowHeight="10755" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Portfolio_Mgmt" sheetId="5" r:id="rId1"/>
@@ -497,31 +497,6 @@
         <rFont val="Arial"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">Valuation Changes: </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="9"/>
-        <color theme="1"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t>IF the market annual return output by valuation model changes materially.</t>
-    </r>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <r>
-      <t xml:space="preserve">- </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="9"/>
-        <color theme="1"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
       <t xml:space="preserve">Market Shifts: </t>
     </r>
     <r>
@@ -1495,6 +1470,31 @@
       <t>When the Projected Portfolio Return falls below the benchmark, it is due to overly conservative cash reserve settings or a lack of eligible opportunities. Manual corrective action is needed to address these issues.</t>
     </r>
     <phoneticPr fontId="17" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">- </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="9"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">Valuation Changes: </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>If the market annual return output by valuation model changes materially.</t>
+    </r>
+    <phoneticPr fontId="2" type="noConversion"/>
   </si>
 </sst>
 </file>
@@ -1950,17 +1950,17 @@
     <xf numFmtId="179" fontId="26" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="4" fontId="6" fillId="5" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -2321,7 +2321,7 @@
   <sheetData>
     <row r="1" spans="1:5">
       <c r="A1" s="20" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
     </row>
     <row r="2" spans="1:5">
@@ -2334,21 +2334,21 @@
       <c r="E2" s="21"/>
     </row>
     <row r="4" spans="1:5" ht="24.4" customHeight="1">
-      <c r="B4" s="65" t="s">
-        <v>208</v>
-      </c>
-      <c r="C4" s="65"/>
-      <c r="D4" s="65"/>
-      <c r="E4" s="65"/>
+      <c r="B4" s="64" t="s">
+        <v>207</v>
+      </c>
+      <c r="C4" s="64"/>
+      <c r="D4" s="64"/>
+      <c r="E4" s="64"/>
     </row>
     <row r="5" spans="1:5">
       <c r="B5" s="24" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
     </row>
     <row r="6" spans="1:5">
       <c r="B6" s="24" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
     </row>
     <row r="8" spans="1:5">
@@ -2356,17 +2356,17 @@
         <v>66</v>
       </c>
       <c r="B8" s="19" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="C8" s="62"/>
     </row>
     <row r="9" spans="1:5">
-      <c r="B9" s="65" t="s">
-        <v>220</v>
-      </c>
-      <c r="C9" s="65"/>
-      <c r="D9" s="65"/>
-      <c r="E9" s="65"/>
+      <c r="B9" s="64" t="s">
+        <v>219</v>
+      </c>
+      <c r="C9" s="64"/>
+      <c r="D9" s="64"/>
+      <c r="E9" s="64"/>
     </row>
     <row r="11" spans="1:5">
       <c r="B11" s="23" t="s">
@@ -2402,26 +2402,26 @@
     </row>
     <row r="16" spans="1:5">
       <c r="B16" s="1" t="s">
+        <v>215</v>
+      </c>
+      <c r="C16" s="4" t="s">
         <v>216</v>
-      </c>
-      <c r="C16" s="4" t="s">
-        <v>217</v>
       </c>
     </row>
     <row r="17" spans="1:5">
       <c r="B17" s="1" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="C17" s="24" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
     </row>
     <row r="18" spans="1:5">
       <c r="B18" s="1" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="C18" s="24" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
     </row>
     <row r="20" spans="1:5">
@@ -2431,7 +2431,7 @@
     </row>
     <row r="21" spans="1:5">
       <c r="B21" s="24" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
     </row>
     <row r="22" spans="1:5">
@@ -2441,7 +2441,7 @@
     </row>
     <row r="23" spans="1:5">
       <c r="B23" s="24" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
     </row>
     <row r="25" spans="1:5">
@@ -2449,18 +2449,18 @@
         <v>67</v>
       </c>
       <c r="B25" s="19" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="C25" s="62"/>
     </row>
     <row r="26" spans="1:5">
       <c r="A26" s="18"/>
-      <c r="B26" s="65" t="s">
-        <v>214</v>
-      </c>
-      <c r="C26" s="65"/>
-      <c r="D26" s="65"/>
-      <c r="E26" s="65"/>
+      <c r="B26" s="64" t="s">
+        <v>213</v>
+      </c>
+      <c r="C26" s="64"/>
+      <c r="D26" s="64"/>
+      <c r="E26" s="64"/>
     </row>
     <row r="27" spans="1:5">
       <c r="A27" s="18"/>
@@ -2468,10 +2468,10 @@
     <row r="28" spans="1:5">
       <c r="A28" s="18"/>
       <c r="B28" s="51" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="C28" s="51" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
     </row>
     <row r="29" spans="1:5">
@@ -2492,15 +2492,15 @@
     </row>
     <row r="32" spans="1:5">
       <c r="B32" s="51" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="C32" s="51" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
     </row>
     <row r="33" spans="1:5">
       <c r="B33" s="26" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="C33" s="60">
         <f>C29-C34</f>
@@ -2509,7 +2509,7 @@
     </row>
     <row r="34" spans="1:5">
       <c r="B34" s="26" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="C34" s="59">
         <v>1</v>
@@ -2554,24 +2554,24 @@
       </c>
     </row>
     <row r="41" spans="1:5">
-      <c r="B41" s="65" t="s">
-        <v>158</v>
-      </c>
-      <c r="C41" s="65"/>
-      <c r="D41" s="65"/>
-      <c r="E41" s="65"/>
+      <c r="B41" s="64" t="s">
+        <v>157</v>
+      </c>
+      <c r="C41" s="64"/>
+      <c r="D41" s="64"/>
+      <c r="E41" s="64"/>
     </row>
     <row r="42" spans="1:5" ht="24.4" customHeight="1">
-      <c r="B42" s="65" t="s">
+      <c r="B42" s="64" t="s">
         <v>88</v>
       </c>
-      <c r="C42" s="65"/>
-      <c r="D42" s="65"/>
-      <c r="E42" s="65"/>
+      <c r="C42" s="64"/>
+      <c r="D42" s="64"/>
+      <c r="E42" s="64"/>
     </row>
     <row r="44" spans="1:5">
       <c r="A44" s="21" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="B44" s="21"/>
       <c r="C44" s="21"/>
@@ -2579,12 +2579,12 @@
       <c r="E44" s="21"/>
     </row>
     <row r="46" spans="1:5">
-      <c r="B46" s="65" t="s">
-        <v>218</v>
-      </c>
-      <c r="C46" s="65"/>
-      <c r="D46" s="65"/>
-      <c r="E46" s="65"/>
+      <c r="B46" s="64" t="s">
+        <v>217</v>
+      </c>
+      <c r="C46" s="64"/>
+      <c r="D46" s="64"/>
+      <c r="E46" s="64"/>
     </row>
     <row r="48" spans="1:5">
       <c r="B48" s="23" t="s">
@@ -2596,7 +2596,7 @@
         <v>94</v>
       </c>
       <c r="C50" s="51" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="D50" s="57"/>
       <c r="E50" s="57"/>
@@ -2629,7 +2629,7 @@
         <v>0.2</v>
       </c>
       <c r="D53" s="63" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="E53" s="56"/>
     </row>
@@ -2719,7 +2719,7 @@
     </row>
     <row r="63" spans="2:5" ht="12" thickBot="1">
       <c r="D63" s="42" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="E63" s="43">
         <f>IF(E62&lt;=2,C51,IF(E62&gt;=6,C53,C52))</f>
@@ -2729,12 +2729,12 @@
     <row r="64" spans="2:5" ht="12" thickTop="1"/>
     <row r="65" spans="1:5">
       <c r="B65" s="23" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
     </row>
     <row r="66" spans="1:5">
       <c r="B66" s="54" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="C66" s="55">
         <f>-E63*(C37-Cash_Yield)</f>
@@ -2743,7 +2743,7 @@
     </row>
     <row r="67" spans="1:5">
       <c r="B67" s="54" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="C67" s="55">
         <f>C37+C66</f>
@@ -2756,7 +2756,7 @@
     </row>
     <row r="69" spans="1:5">
       <c r="B69" s="39" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
     </row>
     <row r="71" spans="1:5">
@@ -2769,223 +2769,223 @@
       <c r="E71" s="21"/>
     </row>
     <row r="73" spans="1:5">
-      <c r="B73" s="65" t="s">
-        <v>201</v>
-      </c>
-      <c r="C73" s="65"/>
-      <c r="D73" s="65"/>
-      <c r="E73" s="65"/>
+      <c r="B73" s="64" t="s">
+        <v>200</v>
+      </c>
+      <c r="C73" s="64"/>
+      <c r="D73" s="64"/>
+      <c r="E73" s="64"/>
     </row>
     <row r="75" spans="1:5">
       <c r="A75" s="28" t="s">
         <v>66</v>
       </c>
       <c r="B75" s="20" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
     </row>
     <row r="76" spans="1:5">
       <c r="B76" s="24" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
     </row>
     <row r="77" spans="1:5">
       <c r="B77" s="24" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
     </row>
     <row r="79" spans="1:5">
       <c r="A79" s="28" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="B79" s="20" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
     </row>
     <row r="80" spans="1:5">
       <c r="B80" s="39" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
     </row>
     <row r="81" spans="1:5">
       <c r="B81" s="24" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
     </row>
     <row r="82" spans="1:5">
       <c r="B82" s="24" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
     </row>
     <row r="83" spans="1:5">
       <c r="B83" s="24" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
     </row>
     <row r="85" spans="1:5">
       <c r="A85" s="28" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="B85" s="20" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
     </row>
     <row r="86" spans="1:5">
       <c r="B86" s="24" t="s">
+        <v>195</v>
+      </c>
+    </row>
+    <row r="87" spans="1:5">
+      <c r="B87" s="67" t="s">
         <v>196</v>
       </c>
-    </row>
-    <row r="87" spans="1:5">
-      <c r="B87" s="66" t="s">
-        <v>197</v>
-      </c>
-      <c r="C87" s="66"/>
-      <c r="D87" s="66"/>
-      <c r="E87" s="66"/>
+      <c r="C87" s="67"/>
+      <c r="D87" s="67"/>
+      <c r="E87" s="67"/>
     </row>
     <row r="88" spans="1:5">
-      <c r="B88" s="64" t="s">
-        <v>195</v>
-      </c>
-      <c r="C88" s="64"/>
-      <c r="D88" s="64"/>
-      <c r="E88" s="64"/>
+      <c r="B88" s="66" t="s">
+        <v>194</v>
+      </c>
+      <c r="C88" s="66"/>
+      <c r="D88" s="66"/>
+      <c r="E88" s="66"/>
     </row>
     <row r="89" spans="1:5" ht="24.4" customHeight="1">
-      <c r="B89" s="65" t="s">
-        <v>194</v>
-      </c>
-      <c r="C89" s="65"/>
-      <c r="D89" s="65"/>
-      <c r="E89" s="65"/>
+      <c r="B89" s="64" t="s">
+        <v>193</v>
+      </c>
+      <c r="C89" s="64"/>
+      <c r="D89" s="64"/>
+      <c r="E89" s="64"/>
     </row>
     <row r="90" spans="1:5">
-      <c r="B90" s="65" t="s">
-        <v>228</v>
-      </c>
-      <c r="C90" s="65"/>
-      <c r="D90" s="65"/>
-      <c r="E90" s="65"/>
+      <c r="B90" s="64" t="s">
+        <v>227</v>
+      </c>
+      <c r="C90" s="64"/>
+      <c r="D90" s="64"/>
+      <c r="E90" s="64"/>
     </row>
     <row r="92" spans="1:5">
       <c r="B92" s="24" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
     </row>
     <row r="93" spans="1:5">
       <c r="B93" s="1" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
     </row>
     <row r="94" spans="1:5">
       <c r="B94" s="61" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
     </row>
     <row r="95" spans="1:5">
       <c r="B95" s="24" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
     </row>
     <row r="96" spans="1:5">
       <c r="B96" s="24" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
     </row>
     <row r="98" spans="1:5">
       <c r="B98" s="24" t="s">
+        <v>220</v>
+      </c>
+    </row>
+    <row r="99" spans="1:5">
+      <c r="B99" s="65" t="s">
         <v>221</v>
       </c>
-    </row>
-    <row r="99" spans="1:5">
-      <c r="B99" s="67" t="s">
-        <v>222</v>
-      </c>
-      <c r="C99" s="67"/>
-      <c r="D99" s="67"/>
-      <c r="E99" s="67"/>
+      <c r="C99" s="65"/>
+      <c r="D99" s="65"/>
+      <c r="E99" s="65"/>
     </row>
     <row r="101" spans="1:5">
       <c r="B101" s="24" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
     </row>
     <row r="102" spans="1:5" ht="12.4">
-      <c r="B102" s="67" t="s">
-        <v>223</v>
-      </c>
-      <c r="C102" s="67"/>
-      <c r="D102" s="67"/>
-      <c r="E102" s="67"/>
+      <c r="B102" s="65" t="s">
+        <v>222</v>
+      </c>
+      <c r="C102" s="65"/>
+      <c r="D102" s="65"/>
+      <c r="E102" s="65"/>
     </row>
     <row r="103" spans="1:5" ht="24.4" customHeight="1">
-      <c r="B103" s="65" t="s">
-        <v>215</v>
-      </c>
-      <c r="C103" s="65"/>
-      <c r="D103" s="65"/>
-      <c r="E103" s="65"/>
+      <c r="B103" s="64" t="s">
+        <v>214</v>
+      </c>
+      <c r="C103" s="64"/>
+      <c r="D103" s="64"/>
+      <c r="E103" s="64"/>
     </row>
     <row r="105" spans="1:5">
       <c r="A105" s="28" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="B105" s="20" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
     </row>
     <row r="106" spans="1:5">
       <c r="B106" s="1" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
     </row>
     <row r="107" spans="1:5">
       <c r="B107" s="1" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
     </row>
     <row r="109" spans="1:5">
       <c r="B109" s="1" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
     </row>
     <row r="110" spans="1:5">
       <c r="B110" s="1" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
     </row>
     <row r="112" spans="1:5">
       <c r="B112" s="23" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
     </row>
     <row r="113" spans="1:5">
       <c r="B113" s="1" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="C113" s="44">
-        <v>0.4</v>
+        <v>0.5490782759805124</v>
       </c>
     </row>
     <row r="114" spans="1:5">
       <c r="B114" s="1" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="C114" s="44">
-        <v>0.13</v>
+        <v>8.956135035007412E-2</v>
       </c>
       <c r="D114" s="62" t="str">
         <f>IF(C114&lt;benchmark,"Warning: Return is lower than the Benchmark.","")</f>
-        <v/>
+        <v>Warning: Return is lower than the Benchmark.</v>
       </c>
     </row>
     <row r="116" spans="1:5" ht="24.4" customHeight="1">
-      <c r="B116" s="65" t="s">
-        <v>229</v>
-      </c>
-      <c r="C116" s="65"/>
-      <c r="D116" s="65"/>
-      <c r="E116" s="65"/>
+      <c r="B116" s="64" t="s">
+        <v>228</v>
+      </c>
+      <c r="C116" s="64"/>
+      <c r="D116" s="64"/>
+      <c r="E116" s="64"/>
     </row>
     <row r="118" spans="1:5">
       <c r="A118" s="21" t="s">
@@ -3008,22 +3008,16 @@
     </row>
     <row r="122" spans="1:5">
       <c r="B122" s="24" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
     </row>
     <row r="123" spans="1:5">
       <c r="B123" s="24" t="s">
-        <v>100</v>
+        <v>229</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="15">
-    <mergeCell ref="B116:E116"/>
-    <mergeCell ref="B99:E99"/>
-    <mergeCell ref="B102:E102"/>
-    <mergeCell ref="B103:E103"/>
-    <mergeCell ref="B89:E89"/>
-    <mergeCell ref="B90:E90"/>
     <mergeCell ref="B88:E88"/>
     <mergeCell ref="B73:E73"/>
     <mergeCell ref="B87:E87"/>
@@ -3033,6 +3027,12 @@
     <mergeCell ref="B26:E26"/>
     <mergeCell ref="B41:E41"/>
     <mergeCell ref="B42:E42"/>
+    <mergeCell ref="B116:E116"/>
+    <mergeCell ref="B99:E99"/>
+    <mergeCell ref="B102:E102"/>
+    <mergeCell ref="B103:E103"/>
+    <mergeCell ref="B89:E89"/>
+    <mergeCell ref="B90:E90"/>
   </mergeCells>
   <phoneticPr fontId="17" type="noConversion"/>
   <pageMargins left="0.25" right="0.25" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -3074,7 +3074,7 @@
       <c r="E1" s="71"/>
       <c r="F1" s="71"/>
       <c r="G1" s="72" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="H1" s="72"/>
       <c r="I1" s="72"/>
@@ -3116,7 +3116,7 @@
         <v>62</v>
       </c>
       <c r="I2" s="7" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="J2" s="8" t="s">
         <v>8</v>
@@ -3145,30 +3145,30 @@
     </row>
     <row r="3" spans="1:17">
       <c r="B3" s="11" t="s">
+        <v>161</v>
+      </c>
+      <c r="C3" s="11" t="s">
         <v>162</v>
       </c>
-      <c r="C3" s="11" t="s">
+      <c r="D3" s="2">
+        <v>15.4</v>
+      </c>
+      <c r="E3" s="12" t="s">
         <v>163</v>
       </c>
-      <c r="D3" s="2">
-        <v>14.94</v>
-      </c>
-      <c r="E3" s="12" t="s">
-        <v>164</v>
-      </c>
       <c r="F3" s="15">
-        <v>0.19401142226230528</v>
+        <v>0.18108249888642258</v>
       </c>
       <c r="G3" s="15">
-        <f t="shared" ref="G3:G5" si="0">F3 - $C$10</f>
-        <v>0.19401142226230528</v>
+        <f t="shared" ref="G3:G5" si="0">F3 - $C$12</f>
+        <v>0.18108249888642258</v>
       </c>
       <c r="H3" s="15">
-        <f t="shared" ref="H3:H5" si="1">F3 - $C$11</f>
-        <v>0.19401142226230528</v>
+        <f t="shared" ref="H3:H5" si="1">F3 - $C$13</f>
+        <v>0.18108249888642258</v>
       </c>
       <c r="I3" s="15">
-        <v>0.3</v>
+        <v>0.27162374832963387</v>
       </c>
       <c r="J3" s="2">
         <v>14.733437767356989</v>
@@ -3177,50 +3177,50 @@
         <v>20.508980461992877</v>
       </c>
       <c r="L3" s="4">
-        <v>0.11566171481724427</v>
+        <v>0.11220688437465126</v>
       </c>
       <c r="M3" s="4">
-        <v>9.1030789825970557E-2</v>
+        <v>8.8311688311688313E-2</v>
       </c>
       <c r="N3" s="13" t="s">
+        <v>164</v>
+      </c>
+      <c r="O3" s="11" t="s">
         <v>165</v>
-      </c>
-      <c r="O3" s="11" t="s">
-        <v>166</v>
       </c>
       <c r="P3" s="14">
         <v>45716</v>
       </c>
       <c r="Q3" s="11" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
     </row>
     <row r="4" spans="1:17">
       <c r="B4" s="11" t="s">
+        <v>167</v>
+      </c>
+      <c r="C4" s="11" t="s">
         <v>168</v>
       </c>
-      <c r="C4" s="11" t="s">
-        <v>169</v>
-      </c>
       <c r="D4" s="2">
-        <v>7.77</v>
+        <v>7.88</v>
       </c>
       <c r="E4" s="12" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="F4" s="15">
-        <v>0.12514862916378067</v>
+        <v>0.11953198379323582</v>
       </c>
       <c r="G4" s="15">
         <f t="shared" si="0"/>
-        <v>0.12514862916378067</v>
+        <v>0.11953198379323582</v>
       </c>
       <c r="H4" s="15">
         <f t="shared" si="1"/>
-        <v>0.12514862916378067</v>
+        <v>0.11953198379323582</v>
       </c>
       <c r="I4" s="15">
-        <v>3.674075125745891E-2</v>
+        <v>0.17929797568985373</v>
       </c>
       <c r="J4" s="2">
         <v>6.4883606756817951</v>
@@ -3229,74 +3229,74 @@
         <v>9.1006872475781417</v>
       </c>
       <c r="L4" s="4">
-        <v>3.975526022937774E-2</v>
+        <v>3.9200301012977792E-2</v>
       </c>
       <c r="M4" s="4">
-        <v>7.4646074646074645E-2</v>
+        <v>7.3604060913705582E-2</v>
       </c>
       <c r="N4" s="13" t="s">
+        <v>169</v>
+      </c>
+      <c r="O4" s="11" t="s">
         <v>170</v>
-      </c>
-      <c r="O4" s="11" t="s">
-        <v>171</v>
       </c>
       <c r="P4" s="14">
         <v>45716</v>
       </c>
       <c r="Q4" s="11" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
     </row>
     <row r="5" spans="1:17">
       <c r="B5" s="11" t="s">
+        <v>171</v>
+      </c>
+      <c r="C5" s="11" t="s">
         <v>172</v>
-      </c>
-      <c r="C5" s="11" t="s">
-        <v>173</v>
       </c>
       <c r="D5" s="2">
         <v>2.15</v>
       </c>
       <c r="E5" s="12" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="F5" s="15">
-        <v>6.9019080849287207E-2</v>
+        <v>6.6927308782200656E-2</v>
       </c>
       <c r="G5" s="15">
         <f t="shared" si="0"/>
-        <v>6.9019080849287207E-2</v>
+        <v>6.6927308782200656E-2</v>
       </c>
       <c r="H5" s="15">
         <f t="shared" si="1"/>
-        <v>6.9019080849287207E-2</v>
+        <v>6.6927308782200656E-2</v>
       </c>
       <c r="I5" s="15">
         <v>0</v>
       </c>
       <c r="J5" s="2">
-        <v>1.5492157922151617</v>
+        <v>1.5407576206248625</v>
       </c>
       <c r="K5" s="2">
-        <v>2.2482528889477993</v>
+        <v>2.2336371684397625</v>
       </c>
       <c r="L5" s="4">
-        <v>2.1918414948495051E-2</v>
+        <v>2.1775925005107808E-2</v>
       </c>
       <c r="M5" s="4">
         <v>5.4790697674418611E-2</v>
       </c>
       <c r="N5" s="13" t="s">
+        <v>173</v>
+      </c>
+      <c r="O5" s="11" t="s">
         <v>174</v>
-      </c>
-      <c r="O5" s="11" t="s">
-        <v>175</v>
       </c>
       <c r="P5" s="14">
         <v>45716</v>
       </c>
       <c r="Q5" s="11" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
     </row>
     <row r="6" spans="1:17">
@@ -5456,7 +5456,7 @@
   <sheetData>
     <row r="1" spans="1:5">
       <c r="B1" s="20" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
     </row>
     <row r="2" spans="1:5">
@@ -5530,7 +5530,7 @@
         <v>25</v>
       </c>
       <c r="C8" s="1">
-        <v>4.3799999999999999E-2</v>
+        <v>4.1700000000000001E-2</v>
       </c>
       <c r="D8" s="1">
         <v>7.4999999999999997E-2</v>
@@ -5723,162 +5723,162 @@
   <sheetData>
     <row r="1" spans="1:4">
       <c r="B1" s="20" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
     </row>
     <row r="2" spans="1:4">
       <c r="A2" s="5"/>
       <c r="B2" s="6" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
     </row>
     <row r="3" spans="1:4">
       <c r="B3" s="73" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="C3" s="73"/>
       <c r="D3" s="73"/>
     </row>
     <row r="5" spans="1:4">
       <c r="B5" s="74" t="s">
-        <v>108</v>
-      </c>
-      <c r="C5" s="67"/>
-      <c r="D5" s="67"/>
+        <v>107</v>
+      </c>
+      <c r="C5" s="65"/>
+      <c r="D5" s="65"/>
     </row>
     <row r="6" spans="1:4">
       <c r="B6" s="74" t="s">
-        <v>109</v>
-      </c>
-      <c r="C6" s="67"/>
-      <c r="D6" s="67"/>
+        <v>108</v>
+      </c>
+      <c r="C6" s="65"/>
+      <c r="D6" s="65"/>
     </row>
     <row r="8" spans="1:4">
       <c r="B8" s="1" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
     </row>
     <row r="10" spans="1:4">
       <c r="A10" s="5"/>
       <c r="B10" s="6" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
     </row>
     <row r="11" spans="1:4">
       <c r="B11" s="73" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="C11" s="73"/>
       <c r="D11" s="73"/>
     </row>
     <row r="12" spans="1:4">
       <c r="B12" s="73" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="C12" s="73"/>
       <c r="D12" s="73"/>
     </row>
     <row r="14" spans="1:4">
       <c r="B14" s="23" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
     </row>
     <row r="16" spans="1:4" ht="12.4">
       <c r="B16" s="30" t="s">
+        <v>120</v>
+      </c>
+      <c r="C16" s="30" t="s">
         <v>121</v>
-      </c>
-      <c r="C16" s="30" t="s">
-        <v>122</v>
       </c>
     </row>
     <row r="17" spans="1:4">
       <c r="B17" s="26" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="C17" s="26" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
     </row>
     <row r="18" spans="1:4">
       <c r="B18" s="26" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="C18" s="26" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
     </row>
     <row r="19" spans="1:4">
       <c r="B19" s="26" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="C19" s="26" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
     </row>
     <row r="20" spans="1:4">
       <c r="B20" s="26" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="C20" s="26" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
     </row>
     <row r="21" spans="1:4">
       <c r="B21" s="26" t="s">
+        <v>135</v>
+      </c>
+      <c r="C21" s="26" t="s">
         <v>136</v>
-      </c>
-      <c r="C21" s="26" t="s">
-        <v>137</v>
       </c>
     </row>
     <row r="22" spans="1:4">
       <c r="B22" s="26" t="s">
+        <v>137</v>
+      </c>
+      <c r="C22" s="26" t="s">
         <v>138</v>
-      </c>
-      <c r="C22" s="26" t="s">
-        <v>139</v>
       </c>
     </row>
     <row r="23" spans="1:4">
       <c r="B23" s="26" t="s">
+        <v>139</v>
+      </c>
+      <c r="C23" s="26" t="s">
         <v>140</v>
-      </c>
-      <c r="C23" s="26" t="s">
-        <v>141</v>
       </c>
     </row>
     <row r="24" spans="1:4">
       <c r="B24" s="26" t="s">
+        <v>144</v>
+      </c>
+      <c r="C24" s="26" t="s">
         <v>145</v>
-      </c>
-      <c r="C24" s="26" t="s">
-        <v>146</v>
       </c>
     </row>
     <row r="25" spans="1:4">
       <c r="B25" s="26" t="s">
+        <v>141</v>
+      </c>
+      <c r="C25" s="26" t="s">
         <v>142</v>
-      </c>
-      <c r="C25" s="26" t="s">
-        <v>143</v>
       </c>
     </row>
     <row r="27" spans="1:4">
       <c r="A27" s="5"/>
       <c r="B27" s="6" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
     </row>
     <row r="28" spans="1:4">
       <c r="B28" s="73" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="C28" s="73"/>
       <c r="D28" s="73"/>
     </row>
     <row r="29" spans="1:4">
       <c r="B29" s="73" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="C29" s="73"/>
       <c r="D29" s="73"/>
@@ -5886,7 +5886,7 @@
     <row r="31" spans="1:4">
       <c r="A31" s="5"/>
       <c r="B31" s="6" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
     </row>
     <row r="32" spans="1:4">
@@ -5894,46 +5894,46 @@
         <v>66</v>
       </c>
       <c r="B32" s="23" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
     </row>
     <row r="33" spans="1:2">
       <c r="B33" s="1" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
     </row>
     <row r="35" spans="1:2">
       <c r="A35" s="28" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="B35" s="23" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
     </row>
     <row r="36" spans="1:2">
       <c r="B36" s="1" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
     </row>
     <row r="38" spans="1:2">
       <c r="A38" s="5"/>
       <c r="B38" s="6" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
     </row>
     <row r="39" spans="1:2">
       <c r="B39" s="24" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
     </row>
     <row r="40" spans="1:2">
       <c r="B40" s="1" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
     </row>
     <row r="41" spans="1:2">
       <c r="B41" s="1" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Updated Monitor and Models
</commit_message>
<xml_diff>
--- a/financial_models/Stock_Monitor.xlsx
+++ b/financial_models/Stock_Monitor.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jerry\PycharmProjects\Invest_Proc_v4\financial_models\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DF47764D-B7A4-4E2A-9646-59377A0122BC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8000EF81-E224-4FB2-A7CC-204CC55A7F4A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="17115" windowHeight="10755" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="33720" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Portfolio_Mgmt" sheetId="5" r:id="rId1"/>
@@ -2194,17 +2194,17 @@
     <xf numFmtId="166" fontId="22" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
     <xf numFmtId="0" fontId="23" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -2240,7 +2240,29 @@
     <cellStyle name="常规 2" xfId="3" xr:uid="{32ADA8AA-F280-4250-ABBF-7E6B9CB799DC}"/>
     <cellStyle name="超链接" xfId="2" builtinId="8"/>
   </cellStyles>
-  <dxfs count="0"/>
+  <dxfs count="3">
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="5" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="9" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="9" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+  </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
     <mruColors>
@@ -2585,12 +2607,12 @@
       <c r="E2" s="21"/>
     </row>
     <row r="4" spans="1:5" ht="24.4" customHeight="1">
-      <c r="B4" s="95" t="s">
+      <c r="B4" s="94" t="s">
         <v>221</v>
       </c>
-      <c r="C4" s="95"/>
-      <c r="D4" s="95"/>
-      <c r="E4" s="95"/>
+      <c r="C4" s="94"/>
+      <c r="D4" s="94"/>
+      <c r="E4" s="94"/>
     </row>
     <row r="6" spans="1:5">
       <c r="A6" s="20" t="s">
@@ -2602,12 +2624,12 @@
       <c r="C6" s="61"/>
     </row>
     <row r="7" spans="1:5">
-      <c r="B7" s="95" t="s">
+      <c r="B7" s="94" t="s">
         <v>209</v>
       </c>
-      <c r="C7" s="95"/>
-      <c r="D7" s="95"/>
-      <c r="E7" s="95"/>
+      <c r="C7" s="94"/>
+      <c r="D7" s="94"/>
+      <c r="E7" s="94"/>
     </row>
     <row r="9" spans="1:5">
       <c r="B9" s="23" t="s">
@@ -2696,12 +2718,12 @@
     </row>
     <row r="24" spans="1:5">
       <c r="A24" s="18"/>
-      <c r="B24" s="95" t="s">
+      <c r="B24" s="94" t="s">
         <v>220</v>
       </c>
-      <c r="C24" s="95"/>
-      <c r="D24" s="95"/>
-      <c r="E24" s="95"/>
+      <c r="C24" s="94"/>
+      <c r="D24" s="94"/>
+      <c r="E24" s="94"/>
     </row>
     <row r="25" spans="1:5">
       <c r="A25" s="18"/>
@@ -2801,20 +2823,20 @@
       </c>
     </row>
     <row r="39" spans="1:5">
-      <c r="B39" s="95" t="s">
+      <c r="B39" s="94" t="s">
         <v>156</v>
       </c>
-      <c r="C39" s="95"/>
-      <c r="D39" s="95"/>
-      <c r="E39" s="95"/>
+      <c r="C39" s="94"/>
+      <c r="D39" s="94"/>
+      <c r="E39" s="94"/>
     </row>
     <row r="40" spans="1:5" ht="46.6" customHeight="1">
-      <c r="B40" s="95" t="s">
+      <c r="B40" s="94" t="s">
         <v>235</v>
       </c>
-      <c r="C40" s="95"/>
-      <c r="D40" s="95"/>
-      <c r="E40" s="95"/>
+      <c r="C40" s="94"/>
+      <c r="D40" s="94"/>
+      <c r="E40" s="94"/>
     </row>
     <row r="42" spans="1:5">
       <c r="A42" s="21" t="s">
@@ -2826,12 +2848,12 @@
       <c r="E42" s="21"/>
     </row>
     <row r="44" spans="1:5">
-      <c r="B44" s="95" t="s">
+      <c r="B44" s="94" t="s">
         <v>208</v>
       </c>
-      <c r="C44" s="95"/>
-      <c r="D44" s="95"/>
-      <c r="E44" s="95"/>
+      <c r="C44" s="94"/>
+      <c r="D44" s="94"/>
+      <c r="E44" s="94"/>
     </row>
     <row r="46" spans="1:5">
       <c r="B46" s="23" t="s">
@@ -3016,12 +3038,12 @@
       <c r="E69" s="21"/>
     </row>
     <row r="71" spans="1:5">
-      <c r="B71" s="95" t="s">
+      <c r="B71" s="94" t="s">
         <v>196</v>
       </c>
-      <c r="C71" s="95"/>
-      <c r="D71" s="95"/>
-      <c r="E71" s="95"/>
+      <c r="C71" s="94"/>
+      <c r="D71" s="94"/>
+      <c r="E71" s="94"/>
     </row>
     <row r="73" spans="1:5">
       <c r="A73" s="28" t="s">
@@ -3083,36 +3105,36 @@
       </c>
     </row>
     <row r="85" spans="1:5">
-      <c r="B85" s="96" t="s">
+      <c r="B85" s="97" t="s">
         <v>192</v>
       </c>
-      <c r="C85" s="96"/>
-      <c r="D85" s="96"/>
-      <c r="E85" s="96"/>
+      <c r="C85" s="97"/>
+      <c r="D85" s="97"/>
+      <c r="E85" s="97"/>
     </row>
     <row r="86" spans="1:5">
-      <c r="B86" s="94" t="s">
+      <c r="B86" s="96" t="s">
         <v>190</v>
       </c>
-      <c r="C86" s="94"/>
-      <c r="D86" s="94"/>
-      <c r="E86" s="94"/>
+      <c r="C86" s="96"/>
+      <c r="D86" s="96"/>
+      <c r="E86" s="96"/>
     </row>
     <row r="87" spans="1:5" ht="24.4" customHeight="1">
-      <c r="B87" s="95" t="s">
+      <c r="B87" s="94" t="s">
         <v>189</v>
       </c>
-      <c r="C87" s="95"/>
-      <c r="D87" s="95"/>
-      <c r="E87" s="95"/>
+      <c r="C87" s="94"/>
+      <c r="D87" s="94"/>
+      <c r="E87" s="94"/>
     </row>
     <row r="88" spans="1:5" ht="24.4" customHeight="1">
-      <c r="B88" s="95" t="s">
+      <c r="B88" s="94" t="s">
         <v>225</v>
       </c>
-      <c r="C88" s="95"/>
-      <c r="D88" s="95"/>
-      <c r="E88" s="95"/>
+      <c r="C88" s="94"/>
+      <c r="D88" s="94"/>
+      <c r="E88" s="94"/>
     </row>
     <row r="90" spans="1:5">
       <c r="B90" s="24" t="s">
@@ -3145,12 +3167,12 @@
       </c>
     </row>
     <row r="97" spans="1:5">
-      <c r="B97" s="97" t="s">
+      <c r="B97" s="95" t="s">
         <v>211</v>
       </c>
-      <c r="C97" s="97"/>
-      <c r="D97" s="97"/>
-      <c r="E97" s="97"/>
+      <c r="C97" s="95"/>
+      <c r="D97" s="95"/>
+      <c r="E97" s="95"/>
     </row>
     <row r="99" spans="1:5">
       <c r="B99" s="24" t="s">
@@ -3158,20 +3180,20 @@
       </c>
     </row>
     <row r="100" spans="1:5" ht="12.4">
-      <c r="B100" s="97" t="s">
+      <c r="B100" s="95" t="s">
         <v>212</v>
       </c>
-      <c r="C100" s="97"/>
-      <c r="D100" s="97"/>
-      <c r="E100" s="97"/>
+      <c r="C100" s="95"/>
+      <c r="D100" s="95"/>
+      <c r="E100" s="95"/>
     </row>
     <row r="101" spans="1:5" ht="58.5" customHeight="1">
-      <c r="B101" s="95" t="s">
+      <c r="B101" s="94" t="s">
         <v>219</v>
       </c>
-      <c r="C101" s="95"/>
-      <c r="D101" s="95"/>
-      <c r="E101" s="95"/>
+      <c r="C101" s="94"/>
+      <c r="D101" s="94"/>
+      <c r="E101" s="94"/>
     </row>
     <row r="103" spans="1:5">
       <c r="A103" s="28" t="s">
@@ -3219,20 +3241,20 @@
         <v>176</v>
       </c>
       <c r="C112" s="44">
-        <v>0.11959137223365987</v>
+        <v>0.11082705639317539</v>
       </c>
       <c r="D112" s="61" t="str">
         <f>IF(C112&lt;benchmark,"Warning: Return is lower than the Benchmark.","")</f>
-        <v/>
+        <v>Warning: Return is lower than the Benchmark.</v>
       </c>
     </row>
     <row r="114" spans="1:5" ht="24.4" customHeight="1">
-      <c r="B114" s="95" t="s">
+      <c r="B114" s="94" t="s">
         <v>217</v>
       </c>
-      <c r="C114" s="95"/>
-      <c r="D114" s="95"/>
-      <c r="E114" s="95"/>
+      <c r="C114" s="94"/>
+      <c r="D114" s="94"/>
+      <c r="E114" s="94"/>
     </row>
     <row r="116" spans="1:5">
       <c r="A116" s="21" t="s">
@@ -3265,12 +3287,6 @@
     </row>
   </sheetData>
   <mergeCells count="15">
-    <mergeCell ref="B114:E114"/>
-    <mergeCell ref="B97:E97"/>
-    <mergeCell ref="B100:E100"/>
-    <mergeCell ref="B101:E101"/>
-    <mergeCell ref="B87:E87"/>
-    <mergeCell ref="B88:E88"/>
     <mergeCell ref="B86:E86"/>
     <mergeCell ref="B71:E71"/>
     <mergeCell ref="B85:E85"/>
@@ -3280,6 +3296,12 @@
     <mergeCell ref="B24:E24"/>
     <mergeCell ref="B39:E39"/>
     <mergeCell ref="B40:E40"/>
+    <mergeCell ref="B114:E114"/>
+    <mergeCell ref="B97:E97"/>
+    <mergeCell ref="B100:E100"/>
+    <mergeCell ref="B101:E101"/>
+    <mergeCell ref="B87:E87"/>
+    <mergeCell ref="B88:E88"/>
   </mergeCells>
   <phoneticPr fontId="17" type="noConversion"/>
   <pageMargins left="0.25" right="0.25" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -3436,30 +3458,30 @@
         <v>160</v>
       </c>
       <c r="F3" s="15">
-        <v>0.22093639979403168</v>
+        <v>0.19063377748254529</v>
       </c>
       <c r="G3" s="15">
         <f>F3 - Portfolio_Mgmt!$C$10</f>
-        <v>0.10353639979403167</v>
+        <v>7.3233777482545281E-2</v>
       </c>
       <c r="H3" s="15">
         <f>F3 - Portfolio_Mgmt!$C$11</f>
-        <v>0.18643639979403168</v>
+        <v>0.15613377748254528</v>
       </c>
       <c r="I3" s="15">
-        <v>0.22093639979403171</v>
+        <v>0.19063377748254529</v>
       </c>
       <c r="J3" s="2">
-        <v>12.76034731937011</v>
+        <v>11.864263383794571</v>
       </c>
       <c r="K3" s="2">
-        <v>25.861790776733326</v>
+        <v>23.893094370273865</v>
       </c>
       <c r="L3" s="2">
-        <v>16.113365751277065</v>
+        <v>14.974073849390802</v>
       </c>
       <c r="M3" s="86">
-        <v>21.933241308816839</v>
+        <v>20.370426628588771</v>
       </c>
       <c r="N3" s="4">
         <v>6.5626579329258014E-2</v>
@@ -3797,7 +3819,7 @@
         <v>8.7843860478168362E-2</v>
       </c>
       <c r="I8" s="15">
-        <v>6.7201415081279747E-2</v>
+        <v>9.7504037392766141E-2</v>
       </c>
       <c r="J8" s="2">
         <v>11.804906901225705</v>
@@ -6313,6 +6335,21 @@
     <mergeCell ref="L1:M1"/>
   </mergeCells>
   <phoneticPr fontId="2" type="noConversion"/>
+  <conditionalFormatting sqref="J3:J1048576">
+    <cfRule type="expression" dxfId="2" priority="1">
+      <formula>J3&gt;D3</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="L3:L1048576">
+    <cfRule type="expression" dxfId="1" priority="4">
+      <formula>L3&gt;D3</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="M3:M1048576">
+    <cfRule type="expression" dxfId="0" priority="2">
+      <formula>D3&gt;M3</formula>
+    </cfRule>
+  </conditionalFormatting>
   <pageMargins left="0.25" right="0.25" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup scale="75" orientation="landscape" r:id="rId1"/>
 </worksheet>
@@ -6686,7 +6723,7 @@
       </c>
       <c r="H4" s="73">
         <f>VLOOKUP(B4,Opportunities!B$3:I$12,8,FALSE)</f>
-        <v>6.7201415081279747E-2</v>
+        <v>9.7504037392766141E-2</v>
       </c>
     </row>
     <row r="5" spans="1:8">
@@ -6770,7 +6807,7 @@
       </c>
       <c r="H7" s="73">
         <f>VLOOKUP(B7,Opportunities!B$3:I$12,8,FALSE)</f>
-        <v>0.22093639979403171</v>
+        <v>0.19063377748254529</v>
       </c>
     </row>
     <row r="8" spans="1:8">
@@ -6837,7 +6874,7 @@
       </c>
       <c r="H12" s="73">
         <f>VLOOKUP(B12,Opportunities!B$3:I$12,8,FALSE)</f>
-        <v>0.22093639979403171</v>
+        <v>0.19063377748254529</v>
       </c>
     </row>
     <row r="13" spans="1:8">
@@ -6960,15 +6997,15 @@
       <c r="B5" s="106" t="s">
         <v>106</v>
       </c>
-      <c r="C5" s="97"/>
-      <c r="D5" s="97"/>
+      <c r="C5" s="95"/>
+      <c r="D5" s="95"/>
     </row>
     <row r="6" spans="1:4">
       <c r="B6" s="106" t="s">
         <v>107</v>
       </c>
-      <c r="C6" s="97"/>
-      <c r="D6" s="97"/>
+      <c r="C6" s="95"/>
+      <c r="D6" s="95"/>
     </row>
     <row r="8" spans="1:4">
       <c r="B8" s="1" t="s">

</xml_diff>